<commit_message>
Classify 2025 Mercury 8291: Coinbase investment, Newstar COGS, unbundle Art Sales.
EPGC Art Sales is matched Berk/mosaics cash only. Coinbase ACH sits on
Investments. Newstar jewelry fabrication is Art Sales COGS. Remaining
EOEB/L5/Fortuna/Erdal/Aysel/Wise/Koziol cash is ASK, not dumped into P&L.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/tax_turbo_parts/Income.xlsx
+++ b/.cursor/scratch/tax_turbo_parts/Income.xlsx
@@ -16,8 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,8 +28,34 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color theme="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Century Gothic"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -35,26 +64,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6EAF8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D5F5E3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -62,19 +76,54 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -441,183 +490,311 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="19.57" customWidth="1" min="1" max="1"/>
+    <col width="16.71" customWidth="1" min="2" max="2"/>
+    <col width="16.86" customWidth="1" min="3" max="3"/>
+    <col width="12.71" customWidth="1" min="4" max="4"/>
+    <col width="12.14" customWidth="1" min="5" max="5"/>
+    <col width="8.710000000000001" customWidth="1" min="6" max="6"/>
+    <col width="11.14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" t="n">
+      <c r="B1" s="1" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C1" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D1" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E1" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="F1" s="3" t="n">
         <v>2024</v>
       </c>
-      <c r="C1" t="n">
+      <c r="G1" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="D1" t="n">
+      <c r="H1" s="3" t="n">
         <v>2025</v>
       </c>
-      <c r="E1" t="n">
+      <c r="I1" s="3" t="n">
         <v>2025</v>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Projected </t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Projected </t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Projected</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Projected</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Income</t>
         </is>
       </c>
+      <c r="B3" s="4" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Hindman / Freeman W-2 (Monarch deposits — reconcile to W-2)</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hindman </t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>92000</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>97876.85000000001</v>
+      </c>
+      <c r="D4" s="6" t="n">
         <v>110000</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" s="4" t="n">
+        <v>115000</v>
+      </c>
+      <c r="F4" s="7" t="n">
         <v>110000</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="G4" s="8" t="n"/>
+      <c r="H4" s="9" t="n">
+        <v>110000</v>
+      </c>
+      <c r="I4" s="10" t="n">
         <v>70618</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>216 N. Oak Park Ave</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>125</v>
+      </c>
+      <c r="D5" s="6" t="n">
         <v>1500</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="7" t="n">
         <v>1500</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="G5" s="8" t="n"/>
+      <c r="H5" s="9" t="n">
         <v>19500</v>
       </c>
+      <c r="I5" s="9" t="n">
+        <v>19500</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>524 Ferdinand Ave #2 (STR platform net)</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>524 Ferdinand Ave #2</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="7" t="n">
         <v>20000</v>
       </c>
-      <c r="D6" t="n">
+      <c r="G6" s="8" t="n"/>
+      <c r="H6" s="9" t="n">
         <v>17000</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="I6" s="9" t="n">
         <v>17086.94</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>GCM / Gates 1099-NEC</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>GCM Boards</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>14000</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>25875</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>14700</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>14700</v>
+      </c>
+      <c r="F7" s="7" t="n">
         <v>16000</v>
       </c>
-      <c r="D7" t="n">
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="9" t="n">
         <v>21500</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="I7" s="9" t="n">
         <v>21500</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Art Sales (net — see Art Sales tab)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Art Sales</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>15000</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>54777.25</v>
+      </c>
+      <c r="F8" s="7" t="n">
         <v>20000</v>
       </c>
-      <c r="D8" t="n">
+      <c r="G8" s="8" t="n"/>
+      <c r="H8" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="I8" s="10" t="n">
+        <v>23055.06</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Megan's Income</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>67000</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>67000</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>74000</v>
+      </c>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="7" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Megan's Income</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+      <c r="G9" s="8" t="n"/>
+      <c r="H9" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D9" t="n">
+      <c r="I9" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="5" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="B10">
+      <c r="B10" s="13">
         <f>SUM(B4:B9)</f>
         <v/>
       </c>
-      <c r="C10">
+      <c r="C10" s="13">
         <f>SUM(C4:C9)</f>
         <v/>
       </c>
-      <c r="D10">
+      <c r="D10" s="13">
         <f>SUM(D4:D9)</f>
         <v/>
       </c>
-      <c r="E10">
+      <c r="E10" s="13">
         <f>SUM(E4:E9)</f>
         <v/>
       </c>
-    </row>
-    <row r="11"/>
+      <c r="F10" s="14">
+        <f>SUM(F4:F9)</f>
+        <v/>
+      </c>
+      <c r="G10" s="15">
+        <f>SUM(G4:G9)</f>
+        <v/>
+      </c>
+      <c r="H10" s="14">
+        <f>SUM(H4:H9)</f>
+        <v/>
+      </c>
+      <c r="I10" s="14">
+        <f>SUM(I4:I9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n"/>
+      <c r="B11" s="4" t="n"/>
+    </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Notes: E4 Monarch paycheck cash ≠ W-2 Box 1. E5 216 Oak Park LTR cash $19500.00 (Delach + Ava co-tenant CONFIRMED + Joan; vacant Oct + half Nov; half-Nov $975 WAIT 8507). E6 PLATFORM STR net LOCKED. E7 GCM 1099-NEC $21,500 on GCM tab only — NOT EPGC Consultant (reimbursements excluded; May 22 CONFIRMED). E8 Art net $0 until Sale 6428 Cost is filled (Sale Price $11,000 on Art Sales, check to Megan). Not tax advice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>2025 Actual: I4 Monarch paycheck cash ≠ W-2 Box 1. I5 216 LTR cash $19,500. I6 524 #2 STR platform net LOCKED. I7 GCM 1099-NEC $21,500. I8 Art net $23,055.06 = MATCHED Mercury deals only (Berk lots $30,000 − $22,944.94 Cost) + seals $1,000 + mosaics $15,000. Excludes Sale 6428 $11,000 until Cost, David Aaron $13,595 (proposed), Erdal/Aysel/EOEB/L5 ASK. Not tax advice.</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>